<commit_message>
feat: add PackingRuleEngine module and update related components
</commit_message>
<xml_diff>
--- a/测试用例一.xlsx
+++ b/测试用例一.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\HeatTreatment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E6880F-7DFD-4986-B5A3-301B1DE2EC59}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00437F38-7C07-4E16-A1EB-E44BC58663BF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
   <si>
     <t>名称</t>
   </si>
@@ -59,9 +59,6 @@
     <t>备注</t>
   </si>
   <si>
-    <t>M0V</t>
-  </si>
-  <si>
     <t>60-62,</t>
   </si>
   <si>
@@ -74,9 +71,6 @@
     <t>圆柱体：填直径(D)+高度(H)</t>
   </si>
   <si>
-    <t>MOV</t>
-  </si>
-  <si>
     <t>58—62,</t>
   </si>
   <si>
@@ -98,9 +92,6 @@
     <t>57-60,</t>
   </si>
   <si>
-    <t>Cr12mov</t>
-  </si>
-  <si>
     <t>H13</t>
   </si>
   <si>
@@ -144,34 +135,6 @@
   </si>
   <si>
     <t>8. 导入后可在预览弹窗中核对数据，确认无误后追加或替换当前列表。</t>
-  </si>
-  <si>
-    <t>客户</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>恒盛实业</t>
-  </si>
-  <si>
-    <t>锐达科技</t>
-  </si>
-  <si>
-    <t>锦程商贸</t>
-  </si>
-  <si>
-    <t xml:space="preserve">卓远工程 </t>
-  </si>
-  <si>
-    <t>鑫源集团</t>
-  </si>
-  <si>
-    <t>明宇物流</t>
-  </si>
-  <si>
-    <t>浩宇智造</t>
-  </si>
-  <si>
-    <t>安信服务</t>
   </si>
   <si>
     <t>模具A</t>
@@ -280,7 +243,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -408,26 +371,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -498,9 +446,6 @@
     <xf numFmtId="49" fontId="5" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
@@ -1670,84 +1615,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.36328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.36328125" style="26" customWidth="1"/>
-    <col min="3" max="6" width="15" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1796875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14" style="1" customWidth="1"/>
-    <col min="10" max="10" width="22" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13" style="1" customWidth="1"/>
-    <col min="13" max="13" width="28" style="1" customWidth="1"/>
-    <col min="14" max="14" width="8.81640625" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.81640625" style="1"/>
+    <col min="2" max="5" width="15" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13" style="1" customWidth="1"/>
+    <col min="12" max="12" width="28" style="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" customHeight="1">
+    <row r="1" spans="1:12" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="22" customHeight="1">
+      <c r="A2" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="4">
+        <v>328</v>
+      </c>
+      <c r="E2" s="4">
+        <v>52</v>
+      </c>
+      <c r="F2" s="6">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="22" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="4">
-        <v>328</v>
-      </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="4">
-        <v>52</v>
-      </c>
-      <c r="G2" s="6">
-        <v>6</v>
-      </c>
-      <c r="H2" s="7">
+      <c r="G2" s="7">
         <v>131.5</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>20</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>12</v>
@@ -1755,451 +1696,416 @@
       <c r="J2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="9" t="s">
+    </row>
+    <row r="3" spans="1:12" ht="22" customHeight="1">
+      <c r="A3" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="4">
+        <v>160</v>
+      </c>
+      <c r="C3" s="4">
+        <v>155</v>
+      </c>
+      <c r="D3" s="4">
+        <v>37</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="11">
+        <v>1</v>
+      </c>
+      <c r="G3" s="12">
+        <v>7</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="22" customHeight="1">
-      <c r="A3" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="30" t="s">
+      <c r="J3" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="22" customHeight="1">
+      <c r="A4" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="4">
+        <v>395</v>
+      </c>
+      <c r="C4" s="4">
+        <v>329</v>
+      </c>
+      <c r="D4" s="4">
+        <v>17</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="11">
+        <v>10</v>
+      </c>
+      <c r="G4" s="12">
+        <v>157</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="22" customHeight="1">
+      <c r="A5" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="4">
+        <v>220</v>
+      </c>
+      <c r="C5" s="4">
+        <v>85</v>
+      </c>
+      <c r="D5" s="4">
+        <v>30</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="11">
+        <v>18</v>
+      </c>
+      <c r="G5" s="12">
+        <v>250.3</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="22" customHeight="1">
+      <c r="A6" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="4">
+        <v>424</v>
+      </c>
+      <c r="C6" s="4">
+        <v>164</v>
+      </c>
+      <c r="D6" s="4">
+        <v>40</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="11">
+        <v>4</v>
+      </c>
+      <c r="G6" s="12">
+        <v>80.5</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="17" customHeight="1">
+      <c r="A7" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="4">
-        <v>160</v>
-      </c>
-      <c r="D3" s="4">
-        <v>155</v>
-      </c>
-      <c r="E3" s="4">
-        <v>37</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="11">
-        <v>1</v>
-      </c>
-      <c r="H3" s="12">
-        <v>7</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="13" t="s">
+      <c r="B7" s="14">
+        <v>120</v>
+      </c>
+      <c r="C7" s="14">
+        <v>105</v>
+      </c>
+      <c r="D7" s="14">
+        <v>24</v>
+      </c>
+      <c r="E7" s="15"/>
+      <c r="F7" s="12">
+        <v>8</v>
+      </c>
+      <c r="G7" s="12">
+        <v>19.3</v>
+      </c>
+      <c r="H7" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="L3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="22" customHeight="1">
-      <c r="A4" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="4">
-        <v>395</v>
-      </c>
-      <c r="D4" s="4">
-        <v>329</v>
-      </c>
-      <c r="E4" s="4">
-        <v>17</v>
-      </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="11">
-        <v>10</v>
-      </c>
-      <c r="H4" s="12">
-        <v>157</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="22" customHeight="1">
-      <c r="A5" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="4">
-        <v>220</v>
-      </c>
-      <c r="D5" s="4">
-        <v>85</v>
-      </c>
-      <c r="E5" s="4">
-        <v>30</v>
-      </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="11">
-        <v>18</v>
-      </c>
-      <c r="H5" s="12">
-        <v>250.3</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="L5" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="22" customHeight="1">
-      <c r="A6" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="4">
-        <v>424</v>
-      </c>
-      <c r="D6" s="4">
-        <v>164</v>
-      </c>
-      <c r="E6" s="4">
-        <v>40</v>
-      </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="11">
-        <v>4</v>
-      </c>
-      <c r="H6" s="12">
-        <v>80.5</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="K6" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="L6" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="17" customHeight="1">
-      <c r="A7" s="33" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="14">
-        <v>120</v>
-      </c>
-      <c r="D7" s="14">
-        <v>105</v>
-      </c>
-      <c r="E7" s="14">
-        <v>24</v>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="12">
-        <v>8</v>
-      </c>
-      <c r="H7" s="12">
-        <v>19.3</v>
-      </c>
       <c r="I7" s="13" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="K7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="17" customHeight="1">
+      <c r="A8" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="16">
+        <v>360</v>
+      </c>
+      <c r="C8" s="16">
+        <v>125</v>
+      </c>
+      <c r="D8" s="16">
+        <v>65</v>
+      </c>
+      <c r="E8" s="17"/>
+      <c r="F8" s="12">
+        <v>2</v>
+      </c>
+      <c r="G8" s="12">
+        <v>42.6</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="17" customHeight="1">
+      <c r="A9" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="16">
+        <v>157</v>
+      </c>
+      <c r="E9" s="16">
+        <v>22</v>
+      </c>
+      <c r="F9" s="18">
+        <v>38</v>
+      </c>
+      <c r="G9" s="18">
+        <v>9.5</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="L9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M7" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="17" customHeight="1">
-      <c r="A8" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="16">
-        <v>360</v>
-      </c>
-      <c r="D8" s="16">
-        <v>125</v>
-      </c>
-      <c r="E8" s="16">
-        <v>65</v>
-      </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="12">
-        <v>2</v>
-      </c>
-      <c r="H8" s="12">
-        <v>42.6</v>
-      </c>
-      <c r="I8" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="M8" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="17" customHeight="1">
-      <c r="A9" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="16">
-        <v>157</v>
-      </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="16">
-        <v>22</v>
-      </c>
-      <c r="G9" s="18">
-        <v>38</v>
-      </c>
-      <c r="H9" s="18">
-        <v>9.5</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="L9" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="17" customHeight="1">
+    </row>
+    <row r="10" spans="1:12" ht="17" customHeight="1">
       <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="12"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="20"/>
       <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="9"/>
-    </row>
-    <row r="11" spans="1:13" ht="17" customHeight="1">
+      <c r="J10" s="13"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" ht="17" customHeight="1">
       <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
+      <c r="B11" s="21"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="12"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="13"/>
       <c r="I11" s="13"/>
       <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="9"/>
-    </row>
-    <row r="12" spans="1:13" ht="14.65" customHeight="1">
+      <c r="K11" s="10"/>
+      <c r="L11" s="9"/>
+    </row>
+    <row r="12" spans="1:12" ht="14.65" customHeight="1">
       <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
       <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="12"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="13"/>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
       <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="24"/>
-    </row>
-    <row r="13" spans="1:13" ht="17" customHeight="1">
+      <c r="L12" s="24"/>
+    </row>
+    <row r="13" spans="1:12" ht="17" customHeight="1">
       <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
+      <c r="B13" s="21"/>
       <c r="C13" s="21"/>
       <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="12"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="13"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="9"/>
-    </row>
-    <row r="14" spans="1:13" ht="17" customHeight="1">
+      <c r="K13" s="10"/>
+      <c r="L13" s="9"/>
+    </row>
+    <row r="14" spans="1:12" ht="17" customHeight="1">
       <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
       <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="12"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="9"/>
-    </row>
-    <row r="15" spans="1:13" ht="17" customHeight="1">
+      <c r="K14" s="10"/>
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:12" ht="17" customHeight="1">
       <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
       <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="12"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="13"/>
       <c r="I15" s="13"/>
       <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="9"/>
-    </row>
-    <row r="16" spans="1:13" ht="17" customHeight="1">
+      <c r="K15" s="10"/>
+      <c r="L15" s="9"/>
+    </row>
+    <row r="16" spans="1:12" ht="17" customHeight="1">
       <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="22"/>
       <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="12"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="9"/>
-    </row>
-    <row r="17" spans="1:13" ht="17" customHeight="1">
+      <c r="K16" s="10"/>
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="1:12" ht="17" customHeight="1">
       <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
+      <c r="B17" s="21"/>
       <c r="C17" s="21"/>
       <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="12"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="13"/>
       <c r="I17" s="13"/>
       <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="9"/>
-    </row>
-    <row r="18" spans="1:13" ht="17" customHeight="1">
+      <c r="K17" s="10"/>
+      <c r="L17" s="9"/>
+    </row>
+    <row r="18" spans="1:12" ht="17" customHeight="1">
       <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="22"/>
       <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="12"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="13"/>
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="9"/>
-    </row>
-    <row r="19" spans="1:13" ht="17" customHeight="1">
+      <c r="K18" s="10"/>
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="1:12" ht="17" customHeight="1">
       <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="21"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="22"/>
       <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="12"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="13"/>
       <c r="I19" s="13"/>
       <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="9"/>
-    </row>
-    <row r="20" spans="1:13" ht="14.65" customHeight="1">
+      <c r="K19" s="10"/>
+      <c r="L19" s="9"/>
+    </row>
+    <row r="20" spans="1:12" ht="14.65" customHeight="1">
       <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="22"/>
       <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="12"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="13"/>
       <c r="I20" s="13"/>
       <c r="J20" s="13"/>
       <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="25"/>
+      <c r="L20" s="25"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -2223,7 +2129,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="17.899999999999999" customHeight="1">
       <c r="A1" s="27" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
@@ -2239,7 +2145,7 @@
     </row>
     <row r="3" spans="1:5" ht="13.5" customHeight="1">
       <c r="A3" s="29" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B3" s="28"/>
       <c r="C3" s="28"/>
@@ -2248,7 +2154,7 @@
     </row>
     <row r="4" spans="1:5" ht="13.5" customHeight="1">
       <c r="A4" s="29" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B4" s="28"/>
       <c r="C4" s="28"/>
@@ -2257,7 +2163,7 @@
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1">
       <c r="A5" s="29" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="28"/>
@@ -2266,7 +2172,7 @@
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1">
       <c r="A6" s="29" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B6" s="28"/>
       <c r="C6" s="28"/>
@@ -2275,7 +2181,7 @@
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1">
       <c r="A7" s="29" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="28"/>
@@ -2284,7 +2190,7 @@
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1">
       <c r="A8" s="29" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B8" s="28"/>
       <c r="C8" s="28"/>
@@ -2293,7 +2199,7 @@
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1">
       <c r="A9" s="29" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
@@ -2302,7 +2208,7 @@
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1">
       <c r="A10" s="29" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B10" s="28"/>
       <c r="C10" s="28"/>
@@ -2311,7 +2217,7 @@
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1">
       <c r="A11" s="29" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B11" s="28"/>
       <c r="C11" s="28"/>
@@ -2320,7 +2226,7 @@
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1">
       <c r="A12" s="29" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B12" s="28"/>
       <c r="C12" s="28"/>
@@ -2329,7 +2235,7 @@
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1">
       <c r="A13" s="29" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -2338,7 +2244,7 @@
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1">
       <c r="A14" s="29" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>

</xml_diff>